<commit_message>
update: 데이터 명세서 data filled
</commit_message>
<xml_diff>
--- a/seonjukim/iM_법인고객_데이터명세서.xlsx
+++ b/seonjukim/iM_법인고객_데이터명세서.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/greenmoster/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\campus4D051\Desktop\yang\oneteam-project\seonjukim\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2F0F43-02F5-8643-8A06-506AD6572FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73EE888E-9A46-465C-AE8E-F1C2C47DEE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="데이터명세서" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="227">
   <si>
     <t>순번</t>
   </si>
@@ -659,6 +659,51 @@
   <si>
     <t>★[iM뱅크] 2026 데이터판매 목록_20260415.pdf
 [별첨1] 2026년 데이터 공급 목록 · 1~2쪽</t>
+  </si>
+  <si>
+    <t>int64</t>
+  </si>
+  <si>
+    <t>str</t>
+  </si>
+  <si>
+    <t>float64</t>
+  </si>
+  <si>
+    <t>미정</t>
+  </si>
+  <si>
+    <t>float64 유지(float32는 경계값 판정이 뒤집힐 수 있음). 평균보다 중앙값 사용; 보유 판정은 요구불예금좌수_ord로만 수행</t>
+  </si>
+  <si>
+    <t>float64 유지(float32는 경계값 판정이 뒤집힐 수 있음). 평균보다 중앙값 사용</t>
+  </si>
+  <si>
+    <t>float64 유지(float32는 경계값 판정이 뒤집힐 수 있음). 평균보다 중앙값 사용; 운전/시설 주택자금대출 컬럼이 완전히 동일한 중복 추출 의심 변수이므로 분석에서 제외</t>
+  </si>
+  <si>
+    <t>제외</t>
+  </si>
+  <si>
+    <t>_ord(0~9) / _mid(구간 대표값) 생성; 기본 계좌로 보유율이 99.45%여서 변별력이 없으므로 분석에서 제외</t>
+  </si>
+  <si>
+    <t>_ord(0~9) / _mid(구간 대표값) 생성</t>
+  </si>
+  <si>
+    <t>_ord(0~9) / _mid(구간 대표값) 생성; 퇴직연금좌수를 포함하는 컬럼이므로 분석에서 제외</t>
+  </si>
+  <si>
+    <t>_ord(0~9) / _mid(구간 대표값) 생성; 하위 9개 좌수의 합계 컬럼이므로 분석에서 제외</t>
+  </si>
+  <si>
+    <t>_ord(0~9) / _mid(구간 대표값) 생성; 운전/시설 주택자금대출 컬럼이 완전히 동일한 중복 추출 의심 변수이므로 분석에서 제외</t>
+  </si>
+  <si>
+    <t>_ord(0~9) / _mid(구간 대표값) 생성; 하위 3개 좌수의 합계 컬럼이므로 분석에서 제외</t>
+  </si>
+  <si>
+    <t>_mid 만들지 말고 _ord 사용</t>
   </si>
 </sst>
 </file>
@@ -674,30 +719,35 @@
       <sz val="10"/>
       <color rgb="FF222222"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF334155"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF243B53"/>
       <name val="Aptos"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -871,10 +921,13 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -889,38 +942,259 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
+      <font>
+        <sz val="10"/>
+        <color rgb="FF222222"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7F9FB"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFAEB8C4"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFAEB8C4"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFAEB8C4"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFAEB8C4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -963,23 +1237,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DataDictionaryTable" displayName="DataDictionaryTable" ref="A1:O71" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DataDictionaryTable" displayName="DataDictionaryTable" ref="A1:O71" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="순번" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="변수명" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="원본 정의" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="변수 역할" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="원본 단위/범주" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="원본 비고" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="실제 dtype" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="결측치수" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="결측률(%)" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="0값수/0범주수" dataDxfId="7"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="0비율(%)" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="고유값수" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="분석상 주의사항" dataDxfId="4"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="전처리/처리방안" dataDxfId="3"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="분석 사용 여부" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="순번" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="변수명" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="원본 정의" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="변수 역할" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="원본 단위/범주" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="원본 비고" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="실제 dtype" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="결측치수" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="결측률(%)" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="0값수/0범주수" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="0비율(%)" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="고유값수" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="분석상 주의사항" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="전처리/처리방안" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="분석 사용 여부" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1181,11 +1455,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="41.6640625" customWidth="1"/>
+    <col min="3" max="3" width="41.69921875" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="32" customWidth="1"/>
@@ -1195,12 +1469,12 @@
     <col min="10" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="42.83203125" customWidth="1"/>
+    <col min="13" max="13" width="42.796875" customWidth="1"/>
     <col min="14" max="14" width="32" customWidth="1"/>
     <col min="15" max="15" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="45.25" customHeight="1">
+    <row r="1" spans="1:15" ht="45.3" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1247,7 +1521,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="61.25" customHeight="1">
+    <row r="2" spans="1:15" ht="61.2" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1266,17 +1540,31 @@
       <c r="F2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
+      <c r="G2" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4">
+        <v>36</v>
+      </c>
       <c r="M2" s="3"/>
       <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-    </row>
-    <row r="3" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O2" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="61.2" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1295,19 +1583,33 @@
       <c r="F3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+      <c r="G3" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
+        <v>15473</v>
+      </c>
       <c r="M3" s="3" t="s">
         <v>25</v>
       </c>
       <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-    </row>
-    <row r="4" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O3" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="61.2" customHeight="1">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1326,19 +1628,33 @@
       <c r="F4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="G4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4">
+        <v>18</v>
+      </c>
       <c r="M4" s="3" t="s">
         <v>30</v>
       </c>
       <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-    </row>
-    <row r="5" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O4" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="61.2" customHeight="1">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1357,17 +1673,31 @@
       <c r="F5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="G5" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>61</v>
+      </c>
       <c r="M5" s="3"/>
       <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-    </row>
-    <row r="6" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O5" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="61.2" customHeight="1">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1386,17 +1716,31 @@
       <c r="F6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
+      <c r="G6" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H6" s="4">
+        <v>12424</v>
+      </c>
+      <c r="I6" s="4">
+        <v>3.39</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
+        <v>5</v>
+      </c>
       <c r="M6" s="3"/>
       <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-    </row>
-    <row r="7" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O6" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="61.2" customHeight="1">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1415,17 +1759,31 @@
       <c r="F7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
+      <c r="G7" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H7" s="4">
+        <v>12424</v>
+      </c>
+      <c r="I7" s="4">
+        <v>3.39</v>
+      </c>
+      <c r="J7" s="4">
+        <v>0</v>
+      </c>
+      <c r="K7" s="4">
+        <v>0</v>
+      </c>
+      <c r="L7" s="4">
+        <v>13</v>
+      </c>
       <c r="M7" s="3"/>
       <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-    </row>
-    <row r="8" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O7" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="61.2" customHeight="1">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1444,19 +1802,33 @@
       <c r="F8" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="G8" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="4">
+        <v>0</v>
+      </c>
+      <c r="J8" s="4">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4">
+        <v>0</v>
+      </c>
+      <c r="L8" s="4">
+        <v>3</v>
+      </c>
       <c r="M8" s="3" t="s">
         <v>44</v>
       </c>
       <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-    </row>
-    <row r="9" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O8" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="61.2" customHeight="1">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1475,17 +1847,31 @@
       <c r="F9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
+      <c r="G9" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
+        <v>0</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4">
+        <v>2</v>
+      </c>
       <c r="M9" s="3"/>
       <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-    </row>
-    <row r="10" spans="1:15" ht="61.25" customHeight="1">
+      <c r="O9" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="61.2" customHeight="1">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1504,19 +1890,35 @@
       <c r="F10" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
+      <c r="G10" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4">
+        <v>41953</v>
+      </c>
+      <c r="K10" s="4">
+        <v>11.46</v>
+      </c>
+      <c r="L10" s="4">
+        <v>562</v>
+      </c>
       <c r="M10" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-    </row>
-    <row r="11" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N10" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="61.2" customHeight="1">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1535,19 +1937,35 @@
       <c r="F11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
+      <c r="G11" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>347219</v>
+      </c>
+      <c r="K11" s="4">
+        <v>94.87</v>
+      </c>
+      <c r="L11" s="4">
+        <v>479</v>
+      </c>
       <c r="M11" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-    </row>
-    <row r="12" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N11" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="61.2" customHeight="1">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1566,19 +1984,35 @@
       <c r="F12" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
+      <c r="G12" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>0</v>
+      </c>
+      <c r="J12" s="4">
+        <v>349564</v>
+      </c>
+      <c r="K12" s="4">
+        <v>95.51</v>
+      </c>
+      <c r="L12" s="4">
+        <v>312</v>
+      </c>
       <c r="M12" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-    </row>
-    <row r="13" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N12" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="61.2" customHeight="1">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1597,19 +2031,35 @@
       <c r="F13" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
+      <c r="G13" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="4">
+        <v>0</v>
+      </c>
+      <c r="J13" s="4">
+        <v>361265</v>
+      </c>
+      <c r="K13" s="4">
+        <v>98.71</v>
+      </c>
+      <c r="L13" s="4">
+        <v>312</v>
+      </c>
       <c r="M13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-    </row>
-    <row r="14" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N13" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="61.2" customHeight="1">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1628,19 +2078,35 @@
       <c r="F14" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
+      <c r="G14" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4">
+        <v>289146</v>
+      </c>
+      <c r="K14" s="4">
+        <v>79</v>
+      </c>
+      <c r="L14" s="4">
+        <v>571</v>
+      </c>
       <c r="M14" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-    </row>
-    <row r="15" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N14" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="61.2" customHeight="1">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1659,19 +2125,35 @@
       <c r="F15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
+      <c r="G15" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4">
+        <v>298191</v>
+      </c>
+      <c r="K15" s="4">
+        <v>81.48</v>
+      </c>
+      <c r="L15" s="4">
+        <v>464</v>
+      </c>
       <c r="M15" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-    </row>
-    <row r="16" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N15" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="61.2" customHeight="1">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1690,19 +2172,35 @@
       <c r="F16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
+      <c r="G16" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0</v>
+      </c>
+      <c r="I16" s="4">
+        <v>0</v>
+      </c>
+      <c r="J16" s="4">
+        <v>222437</v>
+      </c>
+      <c r="K16" s="4">
+        <v>60.78</v>
+      </c>
+      <c r="L16" s="4">
+        <v>352</v>
+      </c>
       <c r="M16" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-    </row>
-    <row r="17" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N16" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="61.2" customHeight="1">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1721,19 +2219,35 @@
       <c r="F17" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
+      <c r="G17" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0</v>
+      </c>
+      <c r="I17" s="4">
+        <v>0</v>
+      </c>
+      <c r="J17" s="4">
+        <v>72988</v>
+      </c>
+      <c r="K17" s="4">
+        <v>19.940000000000001</v>
+      </c>
+      <c r="L17" s="4">
+        <v>559</v>
+      </c>
       <c r="M17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
-    </row>
-    <row r="18" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N17" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="61.2" customHeight="1">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1752,19 +2266,35 @@
       <c r="F18" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
+      <c r="G18" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4">
+        <v>0</v>
+      </c>
+      <c r="J18" s="4">
+        <v>359461</v>
+      </c>
+      <c r="K18" s="4">
+        <v>98.22</v>
+      </c>
+      <c r="L18" s="4">
+        <v>301</v>
+      </c>
       <c r="M18" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-    </row>
-    <row r="19" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N18" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="61.2" customHeight="1">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1783,19 +2313,35 @@
       <c r="F19" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
+      <c r="G19" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0</v>
+      </c>
+      <c r="I19" s="4">
+        <v>0</v>
+      </c>
+      <c r="J19" s="4">
+        <v>364235</v>
+      </c>
+      <c r="K19" s="4">
+        <v>99.52</v>
+      </c>
+      <c r="L19" s="4">
+        <v>265</v>
+      </c>
       <c r="M19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
-    </row>
-    <row r="20" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N19" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="61.2" customHeight="1">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1814,19 +2360,35 @@
       <c r="F20" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
+      <c r="G20" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4">
+        <v>88536</v>
+      </c>
+      <c r="K20" s="4">
+        <v>24.19</v>
+      </c>
+      <c r="L20" s="4">
+        <v>534</v>
+      </c>
       <c r="M20" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
-    </row>
-    <row r="21" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N20" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="61.2" customHeight="1">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1845,19 +2407,35 @@
       <c r="F21" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
+      <c r="G21" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H21" s="4">
+        <v>0</v>
+      </c>
+      <c r="I21" s="4">
+        <v>0</v>
+      </c>
+      <c r="J21" s="4">
+        <v>361651</v>
+      </c>
+      <c r="K21" s="4">
+        <v>98.81</v>
+      </c>
+      <c r="L21" s="4">
+        <v>247</v>
+      </c>
       <c r="M21" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
-    </row>
-    <row r="22" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N21" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="61.2" customHeight="1">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1876,19 +2454,35 @@
       <c r="F22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
+      <c r="G22" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H22" s="4">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4">
+        <v>0</v>
+      </c>
+      <c r="J22" s="4">
+        <v>365701</v>
+      </c>
+      <c r="K22" s="4">
+        <v>99.92</v>
+      </c>
+      <c r="L22" s="4">
+        <v>52</v>
+      </c>
       <c r="M22" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-    </row>
-    <row r="23" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N22" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="61.2" customHeight="1">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1907,19 +2501,35 @@
       <c r="F23" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
+      <c r="G23" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4">
+        <v>0</v>
+      </c>
+      <c r="J23" s="4">
+        <v>357912</v>
+      </c>
+      <c r="K23" s="4">
+        <v>97.79</v>
+      </c>
+      <c r="L23" s="4">
+        <v>294</v>
+      </c>
       <c r="M23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
-    </row>
-    <row r="24" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N23" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="61.2" customHeight="1">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1938,19 +2548,35 @@
       <c r="F24" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
+      <c r="G24" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H24" s="4">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4">
+        <v>0</v>
+      </c>
+      <c r="J24" s="4">
+        <v>362273</v>
+      </c>
+      <c r="K24" s="4">
+        <v>98.98</v>
+      </c>
+      <c r="L24" s="4">
+        <v>348</v>
+      </c>
       <c r="M24" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N24" s="4"/>
-      <c r="O24" s="4"/>
-    </row>
-    <row r="25" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N24" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O24" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="61.2" customHeight="1">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1969,19 +2595,35 @@
       <c r="F25" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
+      <c r="G25" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H25" s="4">
+        <v>0</v>
+      </c>
+      <c r="I25" s="4">
+        <v>0</v>
+      </c>
+      <c r="J25" s="4">
+        <v>342839</v>
+      </c>
+      <c r="K25" s="4">
+        <v>93.67</v>
+      </c>
+      <c r="L25" s="4">
+        <v>317</v>
+      </c>
       <c r="M25" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
-    </row>
-    <row r="26" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N25" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O25" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="61.2" customHeight="1">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -2000,19 +2642,35 @@
       <c r="F26" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
+      <c r="G26" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H26" s="4">
+        <v>0</v>
+      </c>
+      <c r="I26" s="4">
+        <v>0</v>
+      </c>
+      <c r="J26" s="4">
+        <v>252540</v>
+      </c>
+      <c r="K26" s="4">
+        <v>69</v>
+      </c>
+      <c r="L26" s="4">
+        <v>443</v>
+      </c>
       <c r="M26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4"/>
-    </row>
-    <row r="27" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N26" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="61.2" customHeight="1">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -2031,19 +2689,35 @@
       <c r="F27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
+      <c r="G27" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H27" s="4">
+        <v>0</v>
+      </c>
+      <c r="I27" s="4">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4">
+        <v>260324</v>
+      </c>
+      <c r="K27" s="4">
+        <v>71.13</v>
+      </c>
+      <c r="L27" s="4">
+        <v>416</v>
+      </c>
       <c r="M27" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4"/>
-    </row>
-    <row r="28" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N27" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O27" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="61.2" customHeight="1">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -2062,19 +2736,35 @@
       <c r="F28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
+      <c r="G28" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H28" s="4">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4">
+        <v>0</v>
+      </c>
+      <c r="J28" s="4">
+        <v>360930</v>
+      </c>
+      <c r="K28" s="4">
+        <v>98.62</v>
+      </c>
+      <c r="L28" s="4">
+        <v>248</v>
+      </c>
       <c r="M28" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N28" s="4"/>
-      <c r="O28" s="4"/>
-    </row>
-    <row r="29" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N28" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O28" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="61.2" customHeight="1">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -2093,19 +2783,35 @@
       <c r="F29" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
+      <c r="G29" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H29" s="4">
+        <v>0</v>
+      </c>
+      <c r="I29" s="4">
+        <v>0</v>
+      </c>
+      <c r="J29" s="4">
+        <v>365701</v>
+      </c>
+      <c r="K29" s="4">
+        <v>99.92</v>
+      </c>
+      <c r="L29" s="4">
+        <v>52</v>
+      </c>
       <c r="M29" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N29" s="4"/>
-      <c r="O29" s="4"/>
-    </row>
-    <row r="30" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N29" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="O29" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="61.2" customHeight="1">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2124,19 +2830,35 @@
       <c r="F30" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
+      <c r="G30" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H30" s="4">
+        <v>0</v>
+      </c>
+      <c r="I30" s="4">
+        <v>0</v>
+      </c>
+      <c r="J30" s="4">
+        <v>351239</v>
+      </c>
+      <c r="K30" s="4">
+        <v>95.97</v>
+      </c>
+      <c r="L30" s="4">
+        <v>319</v>
+      </c>
       <c r="M30" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4"/>
-    </row>
-    <row r="31" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N30" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O30" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="61.2" customHeight="1">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2155,19 +2877,35 @@
       <c r="F31" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
+      <c r="G31" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H31" s="4">
+        <v>0</v>
+      </c>
+      <c r="I31" s="4">
+        <v>0</v>
+      </c>
+      <c r="J31" s="4">
+        <v>357462</v>
+      </c>
+      <c r="K31" s="4">
+        <v>97.67</v>
+      </c>
+      <c r="L31" s="4">
+        <v>206</v>
+      </c>
       <c r="M31" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N31" s="4"/>
-      <c r="O31" s="4"/>
-    </row>
-    <row r="32" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N31" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O31" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="61.2" customHeight="1">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2186,19 +2924,35 @@
       <c r="F32" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
+      <c r="G32" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H32" s="4">
+        <v>0</v>
+      </c>
+      <c r="I32" s="4">
+        <v>0</v>
+      </c>
+      <c r="J32" s="4">
+        <v>353789</v>
+      </c>
+      <c r="K32" s="4">
+        <v>96.67</v>
+      </c>
+      <c r="L32" s="4">
+        <v>194</v>
+      </c>
       <c r="M32" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N32" s="4"/>
-      <c r="O32" s="4"/>
-    </row>
-    <row r="33" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N32" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="61.2" customHeight="1">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -2217,19 +2971,35 @@
       <c r="F33" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
+      <c r="G33" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H33" s="4">
+        <v>0</v>
+      </c>
+      <c r="I33" s="4">
+        <v>0</v>
+      </c>
+      <c r="J33" s="4">
+        <v>135589</v>
+      </c>
+      <c r="K33" s="4">
+        <v>37.049999999999997</v>
+      </c>
+      <c r="L33" s="4">
+        <v>411</v>
+      </c>
       <c r="M33" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-    </row>
-    <row r="34" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N33" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O33" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" ht="61.2" customHeight="1">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -2248,19 +3018,35 @@
       <c r="F34" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
+      <c r="G34" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H34" s="4">
+        <v>0</v>
+      </c>
+      <c r="I34" s="4">
+        <v>0</v>
+      </c>
+      <c r="J34" s="4">
+        <v>348556</v>
+      </c>
+      <c r="K34" s="4">
+        <v>95.24</v>
+      </c>
+      <c r="L34" s="4">
+        <v>282</v>
+      </c>
       <c r="M34" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N34" s="4"/>
-      <c r="O34" s="4"/>
-    </row>
-    <row r="35" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N34" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O34" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="61.2" customHeight="1">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -2279,19 +3065,35 @@
       <c r="F35" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
+      <c r="G35" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H35" s="4">
+        <v>0</v>
+      </c>
+      <c r="I35" s="4">
+        <v>0</v>
+      </c>
+      <c r="J35" s="4">
+        <v>283064</v>
+      </c>
+      <c r="K35" s="4">
+        <v>77.34</v>
+      </c>
+      <c r="L35" s="4">
+        <v>612</v>
+      </c>
       <c r="M35" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N35" s="4"/>
-      <c r="O35" s="4"/>
-    </row>
-    <row r="36" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N35" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O35" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" ht="61.2" customHeight="1">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -2310,19 +3112,35 @@
       <c r="F36" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4"/>
+      <c r="G36" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H36" s="4">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4">
+        <v>0</v>
+      </c>
+      <c r="J36" s="4">
+        <v>121668</v>
+      </c>
+      <c r="K36" s="4">
+        <v>33.24</v>
+      </c>
+      <c r="L36" s="4">
+        <v>759</v>
+      </c>
       <c r="M36" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N36" s="4"/>
-      <c r="O36" s="4"/>
-    </row>
-    <row r="37" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N36" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O36" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="61.2" customHeight="1">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -2341,19 +3159,35 @@
       <c r="F37" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
+      <c r="G37" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H37" s="4">
+        <v>0</v>
+      </c>
+      <c r="I37" s="4">
+        <v>0</v>
+      </c>
+      <c r="J37" s="4">
+        <v>259654</v>
+      </c>
+      <c r="K37" s="4">
+        <v>70.95</v>
+      </c>
+      <c r="L37" s="4">
+        <v>429</v>
+      </c>
       <c r="M37" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N37" s="4"/>
-      <c r="O37" s="4"/>
-    </row>
-    <row r="38" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N37" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O37" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" ht="61.2" customHeight="1">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -2372,19 +3206,35 @@
       <c r="F38" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="4"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="4"/>
+      <c r="G38" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H38" s="4">
+        <v>0</v>
+      </c>
+      <c r="I38" s="4">
+        <v>0</v>
+      </c>
+      <c r="J38" s="4">
+        <v>339016</v>
+      </c>
+      <c r="K38" s="4">
+        <v>92.63</v>
+      </c>
+      <c r="L38" s="4">
+        <v>387</v>
+      </c>
       <c r="M38" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N38" s="4"/>
-      <c r="O38" s="4"/>
-    </row>
-    <row r="39" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N38" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="61.2" customHeight="1">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -2403,19 +3253,35 @@
       <c r="F39" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="4"/>
+      <c r="G39" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H39" s="4">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4">
+        <v>262589</v>
+      </c>
+      <c r="K39" s="4">
+        <v>71.75</v>
+      </c>
+      <c r="L39" s="4">
+        <v>547</v>
+      </c>
       <c r="M39" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N39" s="4"/>
-      <c r="O39" s="4"/>
-    </row>
-    <row r="40" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N39" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" ht="61.2" customHeight="1">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -2434,19 +3300,35 @@
       <c r="F40" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="4"/>
-      <c r="J40" s="4"/>
-      <c r="K40" s="4"/>
-      <c r="L40" s="4"/>
+      <c r="G40" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H40" s="4">
+        <v>0</v>
+      </c>
+      <c r="I40" s="4">
+        <v>0</v>
+      </c>
+      <c r="J40" s="4">
+        <v>16481</v>
+      </c>
+      <c r="K40" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="L40" s="4">
+        <v>603</v>
+      </c>
       <c r="M40" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N40" s="4"/>
-      <c r="O40" s="4"/>
-    </row>
-    <row r="41" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N40" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O40" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" ht="61.2" customHeight="1">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -2465,19 +3347,35 @@
       <c r="F41" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="4"/>
+      <c r="G41" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H41" s="4">
+        <v>0</v>
+      </c>
+      <c r="I41" s="4">
+        <v>0</v>
+      </c>
+      <c r="J41" s="4">
+        <v>39401</v>
+      </c>
+      <c r="K41" s="4">
+        <v>10.77</v>
+      </c>
+      <c r="L41" s="4">
+        <v>761</v>
+      </c>
       <c r="M41" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N41" s="4"/>
-      <c r="O41" s="4"/>
-    </row>
-    <row r="42" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N41" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O41" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" ht="61.2" customHeight="1">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -2496,19 +3394,35 @@
       <c r="F42" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="G42" s="4"/>
-      <c r="H42" s="4"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="4"/>
+      <c r="G42" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H42" s="4">
+        <v>0</v>
+      </c>
+      <c r="I42" s="4">
+        <v>0</v>
+      </c>
+      <c r="J42" s="4">
+        <v>12649</v>
+      </c>
+      <c r="K42" s="4">
+        <v>3.46</v>
+      </c>
+      <c r="L42" s="4">
+        <v>840</v>
+      </c>
       <c r="M42" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4"/>
-    </row>
-    <row r="43" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N42" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="O42" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" ht="61.2" customHeight="1">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -2527,19 +3441,35 @@
       <c r="F43" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G43" s="4"/>
-      <c r="H43" s="4"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="4"/>
+      <c r="G43" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H43" s="4">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4">
+        <v>2001</v>
+      </c>
+      <c r="K43" s="4">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="L43" s="4">
+        <v>10</v>
+      </c>
       <c r="M43" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N43" s="4"/>
-      <c r="O43" s="4"/>
-    </row>
-    <row r="44" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N43" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="O43" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" ht="61.2" customHeight="1">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -2558,19 +3488,35 @@
       <c r="F44" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G44" s="4"/>
-      <c r="H44" s="4"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="4"/>
+      <c r="G44" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H44" s="4">
+        <v>0</v>
+      </c>
+      <c r="I44" s="4">
+        <v>0</v>
+      </c>
+      <c r="J44" s="4">
+        <v>341698</v>
+      </c>
+      <c r="K44" s="4">
+        <v>93.36</v>
+      </c>
+      <c r="L44" s="4">
+        <v>10</v>
+      </c>
       <c r="M44" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N44" s="4"/>
-      <c r="O44" s="4"/>
-    </row>
-    <row r="45" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N44" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O44" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" ht="61.2" customHeight="1">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -2589,19 +3535,35 @@
       <c r="F45" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G45" s="4"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
+      <c r="G45" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H45" s="4">
+        <v>0</v>
+      </c>
+      <c r="I45" s="4">
+        <v>0</v>
+      </c>
+      <c r="J45" s="4">
+        <v>344621</v>
+      </c>
+      <c r="K45" s="4">
+        <v>94.16</v>
+      </c>
+      <c r="L45" s="4">
+        <v>8</v>
+      </c>
       <c r="M45" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N45" s="4"/>
-      <c r="O45" s="4"/>
-    </row>
-    <row r="46" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N45" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O45" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" ht="61.2" customHeight="1">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -2620,19 +3582,35 @@
       <c r="F46" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-      <c r="J46" s="4"/>
-      <c r="K46" s="4"/>
-      <c r="L46" s="4"/>
+      <c r="G46" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H46" s="4">
+        <v>0</v>
+      </c>
+      <c r="I46" s="4">
+        <v>0</v>
+      </c>
+      <c r="J46" s="4">
+        <v>359338</v>
+      </c>
+      <c r="K46" s="4">
+        <v>98.18</v>
+      </c>
+      <c r="L46" s="4">
+        <v>6</v>
+      </c>
       <c r="M46" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N46" s="4"/>
-      <c r="O46" s="4"/>
-    </row>
-    <row r="47" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N46" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O46" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" ht="61.2" customHeight="1">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -2651,19 +3629,35 @@
       <c r="F47" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="4"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
+      <c r="G47" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H47" s="4">
+        <v>0</v>
+      </c>
+      <c r="I47" s="4">
+        <v>0</v>
+      </c>
+      <c r="J47" s="4">
+        <v>280555</v>
+      </c>
+      <c r="K47" s="4">
+        <v>76.66</v>
+      </c>
+      <c r="L47" s="4">
+        <v>8</v>
+      </c>
       <c r="M47" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N47" s="4"/>
-      <c r="O47" s="4"/>
-    </row>
-    <row r="48" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N47" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" ht="61.2" customHeight="1">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -2682,19 +3676,35 @@
       <c r="F48" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
-      <c r="J48" s="4"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4"/>
+      <c r="G48" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H48" s="4">
+        <v>0</v>
+      </c>
+      <c r="I48" s="4">
+        <v>0</v>
+      </c>
+      <c r="J48" s="4">
+        <v>290205</v>
+      </c>
+      <c r="K48" s="4">
+        <v>79.290000000000006</v>
+      </c>
+      <c r="L48" s="4">
+        <v>5</v>
+      </c>
       <c r="M48" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N48" s="4"/>
-      <c r="O48" s="4"/>
-    </row>
-    <row r="49" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N48" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" ht="61.2" customHeight="1">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -2713,19 +3723,35 @@
       <c r="F49" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4"/>
-      <c r="L49" s="4"/>
+      <c r="G49" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H49" s="4">
+        <v>0</v>
+      </c>
+      <c r="I49" s="4">
+        <v>0</v>
+      </c>
+      <c r="J49" s="4">
+        <v>49415</v>
+      </c>
+      <c r="K49" s="4">
+        <v>13.5</v>
+      </c>
+      <c r="L49" s="4">
+        <v>10</v>
+      </c>
       <c r="M49" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N49" s="4"/>
-      <c r="O49" s="4"/>
-    </row>
-    <row r="50" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N49" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="O49" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" ht="61.2" customHeight="1">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -2744,19 +3770,35 @@
       <c r="F50" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-      <c r="L50" s="4"/>
+      <c r="G50" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H50" s="4">
+        <v>0</v>
+      </c>
+      <c r="I50" s="4">
+        <v>0</v>
+      </c>
+      <c r="J50" s="4">
+        <v>354227</v>
+      </c>
+      <c r="K50" s="4">
+        <v>96.79</v>
+      </c>
+      <c r="L50" s="4">
+        <v>5</v>
+      </c>
       <c r="M50" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N50" s="4"/>
-      <c r="O50" s="4"/>
-    </row>
-    <row r="51" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N50" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O50" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" ht="61.2" customHeight="1">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -2775,19 +3817,35 @@
       <c r="F51" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="4"/>
+      <c r="G51" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H51" s="4">
+        <v>0</v>
+      </c>
+      <c r="I51" s="4">
+        <v>0</v>
+      </c>
+      <c r="J51" s="4">
+        <v>361811</v>
+      </c>
+      <c r="K51" s="4">
+        <v>98.86</v>
+      </c>
+      <c r="L51" s="4">
+        <v>3</v>
+      </c>
       <c r="M51" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N51" s="4"/>
-      <c r="O51" s="4"/>
-    </row>
-    <row r="52" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N51" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O51" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" ht="61.2" customHeight="1">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -2806,19 +3864,35 @@
       <c r="F52" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
-      <c r="I52" s="4"/>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
-      <c r="L52" s="4"/>
+      <c r="G52" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H52" s="4">
+        <v>0</v>
+      </c>
+      <c r="I52" s="4">
+        <v>0</v>
+      </c>
+      <c r="J52" s="4">
+        <v>65811</v>
+      </c>
+      <c r="K52" s="4">
+        <v>17.98</v>
+      </c>
+      <c r="L52" s="4">
+        <v>8</v>
+      </c>
       <c r="M52" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N52" s="4"/>
-      <c r="O52" s="4"/>
-    </row>
-    <row r="53" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N52" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O52" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15" ht="61.2" customHeight="1">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -2837,19 +3911,35 @@
       <c r="F53" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
-      <c r="I53" s="4"/>
-      <c r="J53" s="4"/>
-      <c r="K53" s="4"/>
-      <c r="L53" s="4"/>
+      <c r="G53" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H53" s="4">
+        <v>0</v>
+      </c>
+      <c r="I53" s="4">
+        <v>0</v>
+      </c>
+      <c r="J53" s="4">
+        <v>360725</v>
+      </c>
+      <c r="K53" s="4">
+        <v>98.56</v>
+      </c>
+      <c r="L53" s="4">
+        <v>10</v>
+      </c>
       <c r="M53" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N53" s="4"/>
-      <c r="O53" s="4"/>
-    </row>
-    <row r="54" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N53" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O53" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" ht="61.2" customHeight="1">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -2868,19 +3958,35 @@
       <c r="F54" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-      <c r="I54" s="4"/>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
-      <c r="L54" s="4"/>
+      <c r="G54" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H54" s="4">
+        <v>0</v>
+      </c>
+      <c r="I54" s="4">
+        <v>0</v>
+      </c>
+      <c r="J54" s="4">
+        <v>365679</v>
+      </c>
+      <c r="K54" s="4">
+        <v>99.92</v>
+      </c>
+      <c r="L54" s="4">
+        <v>5</v>
+      </c>
       <c r="M54" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N54" s="4"/>
-      <c r="O54" s="4"/>
-    </row>
-    <row r="55" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N54" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="O54" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" ht="61.2" customHeight="1">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -2899,19 +4005,35 @@
       <c r="F55" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
-      <c r="L55" s="4"/>
+      <c r="G55" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H55" s="4">
+        <v>0</v>
+      </c>
+      <c r="I55" s="4">
+        <v>0</v>
+      </c>
+      <c r="J55" s="4">
+        <v>356828</v>
+      </c>
+      <c r="K55" s="4">
+        <v>97.5</v>
+      </c>
+      <c r="L55" s="4">
+        <v>5</v>
+      </c>
       <c r="M55" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
-    </row>
-    <row r="56" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N55" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O55" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" ht="61.2" customHeight="1">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -2930,19 +4052,35 @@
       <c r="F56" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
-      <c r="L56" s="4"/>
+      <c r="G56" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H56" s="4">
+        <v>0</v>
+      </c>
+      <c r="I56" s="4">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4">
+        <v>359673</v>
+      </c>
+      <c r="K56" s="4">
+        <v>98.27</v>
+      </c>
+      <c r="L56" s="4">
+        <v>4</v>
+      </c>
       <c r="M56" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
-    </row>
-    <row r="57" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N56" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O56" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15" ht="61.2" customHeight="1">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -2961,19 +4099,35 @@
       <c r="F57" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-      <c r="L57" s="4"/>
+      <c r="G57" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H57" s="4">
+        <v>0</v>
+      </c>
+      <c r="I57" s="4">
+        <v>0</v>
+      </c>
+      <c r="J57" s="4">
+        <v>340342</v>
+      </c>
+      <c r="K57" s="4">
+        <v>92.99</v>
+      </c>
+      <c r="L57" s="4">
+        <v>5</v>
+      </c>
       <c r="M57" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
-    </row>
-    <row r="58" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N57" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O57" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" ht="61.2" customHeight="1">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -2992,19 +4146,35 @@
       <c r="F58" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-      <c r="L58" s="4"/>
+      <c r="G58" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H58" s="4">
+        <v>0</v>
+      </c>
+      <c r="I58" s="4">
+        <v>0</v>
+      </c>
+      <c r="J58" s="4">
+        <v>248475</v>
+      </c>
+      <c r="K58" s="4">
+        <v>67.89</v>
+      </c>
+      <c r="L58" s="4">
+        <v>7</v>
+      </c>
       <c r="M58" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N58" s="4"/>
-      <c r="O58" s="4"/>
-    </row>
-    <row r="59" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N58" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="O58" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15" ht="61.2" customHeight="1">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -3023,19 +4193,35 @@
       <c r="F59" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
-      <c r="I59" s="4"/>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4"/>
-      <c r="L59" s="4"/>
+      <c r="G59" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H59" s="4">
+        <v>0</v>
+      </c>
+      <c r="I59" s="4">
+        <v>0</v>
+      </c>
+      <c r="J59" s="4">
+        <v>256334</v>
+      </c>
+      <c r="K59" s="4">
+        <v>70.040000000000006</v>
+      </c>
+      <c r="L59" s="4">
+        <v>6</v>
+      </c>
       <c r="M59" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N59" s="4"/>
-      <c r="O59" s="4"/>
-    </row>
-    <row r="60" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N59" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O59" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" ht="61.2" customHeight="1">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -3054,19 +4240,35 @@
       <c r="F60" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
-      <c r="L60" s="4"/>
+      <c r="G60" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H60" s="4">
+        <v>0</v>
+      </c>
+      <c r="I60" s="4">
+        <v>0</v>
+      </c>
+      <c r="J60" s="4">
+        <v>360447</v>
+      </c>
+      <c r="K60" s="4">
+        <v>98.49</v>
+      </c>
+      <c r="L60" s="4">
+        <v>5</v>
+      </c>
       <c r="M60" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N60" s="4"/>
-      <c r="O60" s="4"/>
-    </row>
-    <row r="61" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N60" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O60" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" ht="61.2" customHeight="1">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -3085,19 +4287,35 @@
       <c r="F61" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G61" s="4"/>
-      <c r="H61" s="4"/>
-      <c r="I61" s="4"/>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
-      <c r="L61" s="4"/>
+      <c r="G61" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H61" s="4">
+        <v>0</v>
+      </c>
+      <c r="I61" s="4">
+        <v>0</v>
+      </c>
+      <c r="J61" s="4">
+        <v>365679</v>
+      </c>
+      <c r="K61" s="4">
+        <v>99.92</v>
+      </c>
+      <c r="L61" s="4">
+        <v>5</v>
+      </c>
       <c r="M61" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N61" s="4"/>
-      <c r="O61" s="4"/>
-    </row>
-    <row r="62" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N61" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="O61" s="4" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" ht="61.2" customHeight="1">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -3116,19 +4334,35 @@
       <c r="F62" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G62" s="4"/>
-      <c r="H62" s="4"/>
-      <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-      <c r="L62" s="4"/>
+      <c r="G62" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H62" s="4">
+        <v>0</v>
+      </c>
+      <c r="I62" s="4">
+        <v>0</v>
+      </c>
+      <c r="J62" s="4">
+        <v>349935</v>
+      </c>
+      <c r="K62" s="4">
+        <v>95.61</v>
+      </c>
+      <c r="L62" s="4">
+        <v>6</v>
+      </c>
       <c r="M62" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N62" s="4"/>
-      <c r="O62" s="4"/>
-    </row>
-    <row r="63" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N62" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O62" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" ht="61.2" customHeight="1">
       <c r="A63" s="3">
         <v>62</v>
       </c>
@@ -3147,19 +4381,35 @@
       <c r="F63" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="4"/>
+      <c r="G63" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H63" s="4">
+        <v>0</v>
+      </c>
+      <c r="I63" s="4">
+        <v>0</v>
+      </c>
+      <c r="J63" s="4">
+        <v>84899</v>
+      </c>
+      <c r="K63" s="4">
+        <v>23.2</v>
+      </c>
+      <c r="L63" s="4">
+        <v>10</v>
+      </c>
       <c r="M63" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="N63" s="4"/>
-      <c r="O63" s="4"/>
-    </row>
-    <row r="64" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N63" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O63" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" ht="61.2" customHeight="1">
       <c r="A64" s="3">
         <v>63</v>
       </c>
@@ -3178,19 +4428,35 @@
       <c r="F64" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="4"/>
+      <c r="G64" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H64" s="4">
+        <v>0</v>
+      </c>
+      <c r="I64" s="4">
+        <v>0</v>
+      </c>
+      <c r="J64" s="4">
+        <v>357462</v>
+      </c>
+      <c r="K64" s="4">
+        <v>97.67</v>
+      </c>
+      <c r="L64" s="4">
+        <v>10</v>
+      </c>
       <c r="M64" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N64" s="4"/>
-      <c r="O64" s="4"/>
-    </row>
-    <row r="65" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N64" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O64" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" ht="61.2" customHeight="1">
       <c r="A65" s="3">
         <v>64</v>
       </c>
@@ -3209,19 +4475,35 @@
       <c r="F65" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G65" s="4"/>
-      <c r="H65" s="4"/>
-      <c r="I65" s="4"/>
-      <c r="J65" s="4"/>
-      <c r="K65" s="4"/>
-      <c r="L65" s="4"/>
+      <c r="G65" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H65" s="4">
+        <v>0</v>
+      </c>
+      <c r="I65" s="4">
+        <v>0</v>
+      </c>
+      <c r="J65" s="4">
+        <v>353794</v>
+      </c>
+      <c r="K65" s="4">
+        <v>96.67</v>
+      </c>
+      <c r="L65" s="4">
+        <v>9</v>
+      </c>
       <c r="M65" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N65" s="4"/>
-      <c r="O65" s="4"/>
-    </row>
-    <row r="66" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N65" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O65" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" ht="61.2" customHeight="1">
       <c r="A66" s="3">
         <v>65</v>
       </c>
@@ -3240,19 +4522,35 @@
       <c r="F66" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G66" s="4"/>
-      <c r="H66" s="4"/>
-      <c r="I66" s="4"/>
-      <c r="J66" s="4"/>
-      <c r="K66" s="4"/>
-      <c r="L66" s="4"/>
+      <c r="G66" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H66" s="4">
+        <v>0</v>
+      </c>
+      <c r="I66" s="4">
+        <v>0</v>
+      </c>
+      <c r="J66" s="4">
+        <v>283064</v>
+      </c>
+      <c r="K66" s="4">
+        <v>77.34</v>
+      </c>
+      <c r="L66" s="4">
+        <v>10</v>
+      </c>
       <c r="M66" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N66" s="4"/>
-      <c r="O66" s="4"/>
-    </row>
-    <row r="67" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N66" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O66" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" ht="61.2" customHeight="1">
       <c r="A67" s="3">
         <v>66</v>
       </c>
@@ -3271,19 +4569,35 @@
       <c r="F67" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G67" s="4"/>
-      <c r="H67" s="4"/>
-      <c r="I67" s="4"/>
-      <c r="J67" s="4"/>
-      <c r="K67" s="4"/>
-      <c r="L67" s="4"/>
+      <c r="G67" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H67" s="4">
+        <v>0</v>
+      </c>
+      <c r="I67" s="4">
+        <v>0</v>
+      </c>
+      <c r="J67" s="4">
+        <v>121668</v>
+      </c>
+      <c r="K67" s="4">
+        <v>33.24</v>
+      </c>
+      <c r="L67" s="4">
+        <v>10</v>
+      </c>
       <c r="M67" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N67" s="4"/>
-      <c r="O67" s="4"/>
-    </row>
-    <row r="68" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N67" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="O67" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" ht="61.2" customHeight="1">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -3302,19 +4616,35 @@
       <c r="F68" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-      <c r="I68" s="4"/>
-      <c r="J68" s="4"/>
-      <c r="K68" s="4"/>
-      <c r="L68" s="4"/>
+      <c r="G68" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H68" s="4">
+        <v>0</v>
+      </c>
+      <c r="I68" s="4">
+        <v>0</v>
+      </c>
+      <c r="J68" s="4">
+        <v>259654</v>
+      </c>
+      <c r="K68" s="4">
+        <v>70.95</v>
+      </c>
+      <c r="L68" s="4">
+        <v>10</v>
+      </c>
       <c r="M68" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N68" s="4"/>
-      <c r="O68" s="4"/>
-    </row>
-    <row r="69" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N68" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O68" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" ht="61.2" customHeight="1">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -3333,19 +4663,35 @@
       <c r="F69" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G69" s="4"/>
-      <c r="H69" s="4"/>
-      <c r="I69" s="4"/>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="4"/>
+      <c r="G69" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H69" s="4">
+        <v>0</v>
+      </c>
+      <c r="I69" s="4">
+        <v>0</v>
+      </c>
+      <c r="J69" s="4">
+        <v>339016</v>
+      </c>
+      <c r="K69" s="4">
+        <v>92.63</v>
+      </c>
+      <c r="L69" s="4">
+        <v>10</v>
+      </c>
       <c r="M69" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N69" s="4"/>
-      <c r="O69" s="4"/>
-    </row>
-    <row r="70" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N69" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O69" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" ht="61.2" customHeight="1">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -3364,19 +4710,35 @@
       <c r="F70" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G70" s="4"/>
-      <c r="H70" s="4"/>
-      <c r="I70" s="4"/>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="4"/>
+      <c r="G70" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H70" s="4">
+        <v>0</v>
+      </c>
+      <c r="I70" s="4">
+        <v>0</v>
+      </c>
+      <c r="J70" s="4">
+        <v>262589</v>
+      </c>
+      <c r="K70" s="4">
+        <v>71.75</v>
+      </c>
+      <c r="L70" s="4">
+        <v>10</v>
+      </c>
       <c r="M70" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N70" s="4"/>
-      <c r="O70" s="4"/>
-    </row>
-    <row r="71" spans="1:15" ht="61.25" customHeight="1">
+      <c r="N70" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O70" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="61.2" customHeight="1">
       <c r="A71" s="3">
         <v>70</v>
       </c>
@@ -3395,22 +4757,38 @@
       <c r="F71" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="G71" s="4"/>
-      <c r="H71" s="4"/>
-      <c r="I71" s="4"/>
-      <c r="J71" s="4"/>
-      <c r="K71" s="4"/>
-      <c r="L71" s="4"/>
+      <c r="G71" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H71" s="4">
+        <v>0</v>
+      </c>
+      <c r="I71" s="4">
+        <v>0</v>
+      </c>
+      <c r="J71" s="4">
+        <v>16481</v>
+      </c>
+      <c r="K71" s="4">
+        <v>4.5</v>
+      </c>
+      <c r="L71" s="4">
+        <v>10</v>
+      </c>
       <c r="M71" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="N71" s="4"/>
-      <c r="O71" s="4"/>
+      <c r="N71" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O71" s="4" t="s">
+        <v>215</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="11" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="O2:O71" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="O2:O71" xr:uid="{6862A3D1-09C8-4DD7-8968-33C30ACD72AF}">
       <formula1>"사용,보류,제외,미정"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3424,116 +4802,116 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="54.83203125" customWidth="1"/>
+    <col min="1" max="1" width="54.796875" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="45.25" customHeight="1">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:2" ht="45.3" customHeight="1">
+      <c r="A1" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="8"/>
-    </row>
-    <row r="2" spans="1:2" ht="64" customHeight="1">
-      <c r="A2" s="9" t="s">
+      <c r="B1" s="10"/>
+    </row>
+    <row r="2" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A2" s="8" t="s">
         <v>131</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="64" customHeight="1">
-      <c r="A3" s="9" t="s">
+    <row r="3" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A3" s="8" t="s">
         <v>133</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="64" customHeight="1">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>135</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="64" customHeight="1">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>137</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="64" customHeight="1">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A6" s="8" t="s">
         <v>139</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="64" customHeight="1">
-      <c r="A7" s="9" t="s">
+    <row r="7" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A7" s="8" t="s">
         <v>141</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="64" customHeight="1">
-      <c r="A8" s="9" t="s">
+    <row r="8" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A8" s="8" t="s">
         <v>143</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="64" customHeight="1">
-      <c r="A9" s="9" t="s">
+    <row r="9" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A9" s="8" t="s">
         <v>145</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="64" customHeight="1">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A10" s="8" t="s">
         <v>147</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="64" customHeight="1">
-      <c r="A11" s="9" t="s">
+    <row r="11" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A11" s="8" t="s">
         <v>149</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="64" customHeight="1">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A12" s="8" t="s">
         <v>151</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="64" customHeight="1">
-      <c r="A13" s="9" t="s">
+    <row r="13" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A13" s="8" t="s">
         <v>153</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="64" customHeight="1">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A14" s="8" t="s">
         <v>155</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -3544,11 +4922,11 @@
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="1:2" ht="45.25" customHeight="1">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:2" ht="45.3" customHeight="1">
+      <c r="A16" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="12"/>
     </row>
     <row r="17" spans="1:2" ht="42.75" customHeight="1">
       <c r="A17" s="5" t="s">
@@ -3558,7 +4936,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="33.25" customHeight="1">
+    <row r="18" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A18" s="3" t="s">
         <v>160</v>
       </c>
@@ -3566,7 +4944,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="33.25" customHeight="1">
+    <row r="19" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>162</v>
       </c>
@@ -3574,7 +4952,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="33.25" customHeight="1">
+    <row r="20" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>164</v>
       </c>
@@ -3582,7 +4960,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="33.25" customHeight="1">
+    <row r="21" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>166</v>
       </c>
@@ -3590,7 +4968,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="33.25" customHeight="1">
+    <row r="22" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>168</v>
       </c>
@@ -3598,7 +4976,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="33.25" customHeight="1">
+    <row r="23" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A23" s="3" t="s">
         <v>170</v>
       </c>
@@ -3606,7 +4984,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="33.25" customHeight="1">
+    <row r="24" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A24" s="3" t="s">
         <v>172</v>
       </c>
@@ -3614,7 +4992,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="33.25" customHeight="1">
+    <row r="25" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>174</v>
       </c>
@@ -3622,7 +5000,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="33.25" customHeight="1">
+    <row r="26" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A26" s="3" t="s">
         <v>176</v>
       </c>
@@ -3630,7 +5008,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="33.25" customHeight="1">
+    <row r="27" spans="1:2" ht="33.299999999999997" customHeight="1">
       <c r="A27" s="3" t="s">
         <v>178</v>
       </c>
@@ -3642,61 +5020,61 @@
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="1:2" ht="64" customHeight="1">
-      <c r="A29" s="9" t="s">
+    <row r="29" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A29" s="8" t="s">
         <v>180</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="64" customHeight="1">
-      <c r="A30" s="9" t="s">
+    <row r="30" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A30" s="8" t="s">
         <v>182</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="64" customHeight="1">
-      <c r="A31" s="9" t="s">
+    <row r="31" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A31" s="8" t="s">
         <v>184</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="64" customHeight="1">
-      <c r="A32" s="9" t="s">
+    <row r="32" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A32" s="8" t="s">
         <v>186</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="64" customHeight="1">
-      <c r="A33" s="9" t="s">
+    <row r="33" spans="1:2" ht="64.05" customHeight="1">
+      <c r="A33" s="8" t="s">
         <v>188</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="45.25" customHeight="1">
-      <c r="A35" s="12" t="s">
+    <row r="35" spans="1:2" ht="45.3" customHeight="1">
+      <c r="A35" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="B35" s="13"/>
-    </row>
-    <row r="36" spans="1:2" ht="40" customHeight="1">
-      <c r="A36" s="14" t="s">
+      <c r="B35" s="14"/>
+    </row>
+    <row r="36" spans="1:2" ht="40.049999999999997" customHeight="1">
+      <c r="A36" s="9" t="s">
         <v>191</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="40" customHeight="1">
+    <row r="37" spans="1:2" ht="40.049999999999997" customHeight="1">
       <c r="A37" s="6" t="s">
         <v>193</v>
       </c>
@@ -3760,24 +5138,24 @@
         <v>206</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="45.25" customHeight="1">
-      <c r="A45" s="14" t="s">
+    <row r="45" spans="1:2" ht="45.3" customHeight="1">
+      <c r="A45" s="9" t="s">
         <v>208</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="69.25" customHeight="1">
-      <c r="A46" s="14" t="s">
+    <row r="46" spans="1:2" ht="69.3" customHeight="1">
+      <c r="A46" s="9" t="s">
         <v>180</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="69.25" customHeight="1">
-      <c r="A47" s="14" t="s">
+    <row r="47" spans="1:2" ht="69.3" customHeight="1">
+      <c r="A47" s="9" t="s">
         <v>188</v>
       </c>
       <c r="B47" s="7" t="s">

</xml_diff>